<commit_message>
+ Balance skill for The Boy Sage.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -6594,7 +6594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C285"/>
+  <dimension ref="A1:C286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38.85546875" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
@@ -11148,12 +11148,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Max HP increases by {0}%. Additionally, initial damage taken is reduced by 18%, increasing by an additional 2% reduction per subsequent hit taken, stacking up to 4 times.</t>
+          <t>Max HP increases by {0}%. Additionally, damage taken is reduced by 15% on the first hit; subsequent hits have a 40% chance to trigger the [Damage Reduced] effect (reducing damage by 10%).</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>HP Tối Đa tăng {0}%. Đồng thời giảm 18% sát thương nhận vào ở lần đầu tiên, mỗi lần chịu đòn sau đó giảm thêm 2%, tối đa cộng dồn 4 lần.</t>
+          <t>HP Tối Đa tăng {0}%. Đồng thời giảm 15% sát thương nhận vào ở đòn đánh đầu tiên; các đòn tiếp theo có 40% tỉ lệ kích hoạt hiệu ứng [Giảm Sát Thương] (giảm 10% sát thương).</t>
         </is>
       </c>
     </row>
@@ -11296,7 +11296,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>STR_LINGLONG_PAGODA_DES</t>
+          <t>STR_FERROUS_CHAOS_DES</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -11313,102 +11313,119 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>STR_LINGLONG_PAGODA_SKILL</t>
+          <t>STR_FERROUS_CHAOS_SKILL</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Increases ATK and DEF by {0}%.When HP &gt; 50%: Increases Skill DMG by 16%.When HP ≤ 50%: Converts 16% of damage dealt into HP recovery.</t>
+          <t>Increases ATK by {0}% and DEF by {0}%. In Overpower state (HP &gt; 50%), increases Skill Damage by 16%. In Bloodbath state (HP ≤ 50%), gains 16% Lifesteal.</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng.Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
+          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>STR_FERROUS_CHAOS_SKILL</t>
+          <t>STR_COOLDOWN_REDUCED</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Increases ATK by {0}% and DEF by {0}%. In Overpower state (HP &gt; 50%), increases Skill Damage by 16%. In Bloodbath state (HP ≤ 50%), gains 16% Lifesteal.</t>
+          <t>-1 CD</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tấn Công và {0}% Phòng Thủ. Trạng thái Áp Đảo (HP &gt; 50%) tăng 16% Sát thương Kỹ năng. Trạng thái Huyết Chiến (HP ≤ 50%) nhận 16% Hút Máu tương đương 16% tổng sát thương gây ra.</t>
+          <t>-1 Hồi Chiêu</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>STR_COOLDOWN_REDUCED</t>
+          <t>STR_NEZHA_ULT_PASSIVE</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>-1 CD</t>
+          <t>When defeating an enemy with Ultimate, activates [Battlefield Sweep], attacking another enemy for 120% ATK.</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>-1 Hồi Chiêu</t>
+          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>STR_NEZHA_ULT_PASSIVE</t>
+          <t>STR_SWEEP_ATTACK</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>When defeating an enemy with Ultimate, activates [Battlefield Sweep], attacking another enemy for 120% ATK.</t>
+          <t>Sweep</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Khi kết liễu kẻ địch bằng chiêu cuối, kích hoạt hiệu ứng [Càn Quét] tấn công 1 kẻ địch khác với 120% ATK.</t>
+          <t>Càn Quét</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>STR_SWEEP_ATTACK</t>
+          <t>STR_PURSUIT_ATTACK</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Sweep</t>
+          <t>Pursuit!</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Càn Quét</t>
+          <t>Truy Kích!</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>STR_PURSUIT_ATTACK</t>
+          <t>STR_DAMAGE_REDUCED</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Pursuit!</t>
+          <t>Damage Reduced!</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Truy Kích!</t>
+          <t>Giảm Sát Thương!</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>STR_THEBOYSAGE_ULTIMATE_PASSIVE</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Ultimate ignores 30% of target's DEF.</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Tuyệt kỹ bỏ qua 30% Phòng Thủ của mục tiêu.</t>
         </is>
       </c>
     </row>
@@ -11429,7 +11446,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34.28515625" customWidth="1" style="6" min="1" max="1"/>
-    <col width="7.7109375" customWidth="1" style="6" min="2" max="2"/>
+    <col width="7.28515625" customWidth="1" style="6" min="2" max="2"/>
     <col width="193.5703125" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -12116,9 +12133,14 @@
           <t>TheBoySage_B_Name</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Fire Spear Strike</t>
+        </is>
+      </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Kĩ năng X</t>
+          <t>Hỏa Tiêm Thương Kích</t>
         </is>
       </c>
     </row>
@@ -12128,9 +12150,14 @@
           <t>TheBoySage_M_Name</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>True Samadhi Fireball</t>
+        </is>
+      </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Kĩ năng X</t>
+          <t>Tam Muội Hỏa Cầu</t>
         </is>
       </c>
     </row>
@@ -12140,9 +12167,14 @@
           <t>TheBoySage_U_Name</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Blazing Meteor Extinction</t>
+        </is>
+      </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Kĩ năng X</t>
+          <t>Thiên Hỏa Phần Thiên</t>
         </is>
       </c>
     </row>
@@ -12152,9 +12184,14 @@
           <t>TheBoySage_B_Des</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Wields the blazing Fire Spear to pierce the target, dealing {0}% ATK damage to a single enemy.</t>
+        </is>
+      </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Kĩ năng X</t>
+          <t>Múa Hỏa Tiêm Thương rực lửa đâm xuyên mục tiêu, gây Sát Thương bằng {0}% Tấn Công lên một kẻ địch.</t>
         </is>
       </c>
     </row>
@@ -12164,9 +12201,14 @@
           <t>TheBoySage_M_Des</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Condenses Samadhi True Fire to launch a blazing fireball, dealing {0}% ATK damage to a single enemy and inflicting 1 stack of [Burn] lasting 2 turns.</t>
+        </is>
+      </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Kĩ năng X</t>
+          <t>Ngưng tụ Tam Muội Chân Hỏa bắn ra quả cầu lửa rực cháy, gây Sát Thương bằng {0}% Tấn Công lên một kẻ địch đồng thời tích thêm 1 tầng [Thiêu Đốt] duy trì 2 hiệp.</t>
         </is>
       </c>
     </row>
@@ -12176,9 +12218,14 @@
           <t>TheBoySage_U_Des</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Summons a colossal flaming meteor from the heavens to strike down, dealing {0}% ATK damage. The attack ignores {1}% of target's DEF and inflicts 1 stack of [Burn] lasting 2 turns.</t>
+        </is>
+      </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Kĩ năng X</t>
+          <t>Triệu hồi một quả cầu thiên thạch lửa khổng lồ từ trên trời giáng xuống, gây Sát Thương bằng {0}% Tấn Công. Đòn đánh bỏ qua {1}% Phòng Thủ đồng thời tích thêm 1 tầng [Thiêu Đốt] duy trì 2 hiệp.</t>
         </is>
       </c>
     </row>
@@ -12655,7 +12702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
@@ -13011,6 +13058,40 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EFF_BURN_NAME</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Burn</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Thiêu Đốt</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>EFF_BURN_DES</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Takes damage equal to {0}% Max HP each turn for {1} turns.</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Mỗi hiệp chịu sát thương bằng {0}% Máu Tối Đa, duy trì {1} hiệp.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
+ Fix bug weapon add shield
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -7426,12 +7426,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Increases SPEED by {0}% and ATK by {1}%. Increases the effectiveness of Enhancement and Support skills by {2}%.</t>
+          <t>Increases SPEED by {0}% and ATK by {1}%. Increases the effectiveness of Enhancement, Support, and Shield skills by {2}%.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Tăng {0}% Tốc Độ và {1}% Tấn Công. Tăng thêm {2}% hiệu quả cho các kỹ năng Cường Hóa và Hỗ Trợ.</t>
+          <t>Tăng {0}% Tốc Độ và {1}% Tấn Công. Tăng thêm {2}% hiệu quả cho các kỹ năng Cường Hóa, Hỗ Trợ và Tạo Khiên.</t>
         </is>
       </c>
     </row>
@@ -7528,12 +7528,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Increases HP by {0}% and DEF by {1}%. Increases the effectiveness of Healing skills by {2}%.</t>
+          <t>Increases HP by {0}% and DEF by {1}%. Increases the effectiveness of Healing and Shield skills by {2}%.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tăng {0}% HP và {1}% Phòng Thủ. Tăng thêm {2}% hiệu quả cho các kỹ năng Hồi Máu.</t>
+          <t>Tăng {0}% HP và {1}% Phòng Thủ. Tăng thêm {2}% hiệu quả cho các kỹ năng Hồi Máu và Tạo Khiên.</t>
         </is>
       </c>
     </row>
@@ -12348,12 +12348,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Swings the dragon blade forward, dealing {0}% ATK to an enemy with 30% built-in Armor Penetration.</t>
+          <t>Swings the dragon blade forward, dealing {0}% ATK to an enemy with 15% built-in Armor Penetration.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Vung bảo kiếm chém dứt khoát về phía trước, gây ST bằng {0}% Tấn Công cho một kẻ địch. Đòn đánh có sẵn 30% Phòng Thủ.</t>
+          <t>Vung bảo kiếm chém dứt khoát về phía trước, gây ST bằng {0}% Tấn Công cho một kẻ địch. Đòn đánh có sẵn 15% Xuyên Giáp.</t>
         </is>
       </c>
     </row>
@@ -12365,12 +12365,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Summons thunder dragon energy to blast a lightning orb, dealing {0}% ATK to an enemy and grants self [Gale Chase], increasing Speed by 30% for 2 turns.</t>
+          <t>Summons thunder dragon energy to blast a lightning orb, dealing {0}% ATK to an enemy and grants self [Gale Chase], increasing Speed by 15% for 2 turns.</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Triệu hồi Lôi Long ngưng tụ và bắn quả cầu sét về phía mục tiêu, gây ST bằng {0}% Tấn Công cho một kẻ địch, đồng thời bản thân lập tức nhận trạng thái [Truy Phong] - Tăng 30% Tốc Độ trong 2 hiệp.</t>
+          <t>Triệu hồi Lôi Long ngưng tụ và bắn quả cầu sét về phía mục tiêu, gây ST bằng {0}% Tấn Công cho một kẻ địch, đồng thời bản thân lập tức nhận trạng thái [Truy Phong] - Tăng 15% Tốc Độ trong 2 hiệp.</t>
         </is>
       </c>
     </row>

</xml_diff>